<commit_message>
Changed N notation to NT.
</commit_message>
<xml_diff>
--- a/homeworks/2/homework2_branch_2bit_bht.xlsx
+++ b/homeworks/2/homework2_branch_2bit_bht.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\github\cs1541\CS1541_Source\homeworks\2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\github\cs2410\CS2410_Spring2026\homeworks\2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E9D4630-AB8C-4648-83B2-B3F6CF7932F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABD4750E-4CC0-4854-83D4-B914750192D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1665" yWindow="4410" windowWidth="27135" windowHeight="11070" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,9 +33,6 @@
     <t>T</t>
   </si>
   <si>
-    <t>N</t>
-  </si>
-  <si>
     <t>2-bit state</t>
   </si>
   <si>
@@ -52,6 +49,9 @@
   </si>
   <si>
     <t>n</t>
+  </si>
+  <si>
+    <t>NT</t>
   </si>
 </sst>
 </file>
@@ -413,36 +413,36 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -455,10 +455,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -472,10 +472,10 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>

</xml_diff>